<commit_message>
Actualizacao da 2 sessao
</commit_message>
<xml_diff>
--- a/log_acoes.xlsx
+++ b/log_acoes.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -419,6 +419,23 @@
       <c r="C4" t="inlineStr">
         <is>
           <t>2026-02-19 11:47:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Atualizou os dados</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2026-02-23 11:27:05</t>
         </is>
       </c>
     </row>
@@ -683,13 +700,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4E2D3D11-3789-428C-89E4-60021E5080D6}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{13A4FD71-B37F-456A-AE88-1DAE0EA9F817}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A4B53037-D293-4797-8EC7-AE2F089A049B}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BC2F6531-8991-4EF1-B5FD-02938A64FDD3}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0262BBF7-7C5E-43E5-B11A-B7A6A5D83CAA}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B90CB467-6C5A-4122-A080-C4EB558C3D2A}"/>
 </file>
</xml_diff>

<commit_message>
Actualizacao da sessao 2
</commit_message>
<xml_diff>
--- a/log_acoes.xlsx
+++ b/log_acoes.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -436,6 +436,40 @@
       <c r="C5" t="inlineStr">
         <is>
           <t>2026-02-23 11:27:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Atualizou os dados</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2026-02-24 15:22:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Atualizou os dados</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2026-02-24 16:15:34</t>
         </is>
       </c>
     </row>
@@ -700,13 +734,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{13A4FD71-B37F-456A-AE88-1DAE0EA9F817}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{45CFDEC3-A1A7-49EB-9FB6-F7C16EFB765E}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BC2F6531-8991-4EF1-B5FD-02938A64FDD3}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8CF03338-996D-4081-9BE1-83A5DEE77CC6}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B90CB467-6C5A-4122-A080-C4EB558C3D2A}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FE22F1CB-2E0B-4D9B-8219-06F2063522A5}"/>
 </file>
</xml_diff>

<commit_message>
Desenvolvimento da Pagina Qualidade das sessoes
</commit_message>
<xml_diff>
--- a/log_acoes.xlsx
+++ b/log_acoes.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -640,6 +640,57 @@
       <c r="C17" t="inlineStr">
         <is>
           <t>2026-03-19 14:20:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Atualizou os dados</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>2026-03-20 11:30:25</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Atualizou os dados</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>2026-03-24 10:28:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Atualizou os dados</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>2026-03-24 10:37:25</t>
         </is>
       </c>
     </row>
@@ -904,13 +955,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BCE9CECD-6B82-46B1-92A1-9CE773CCA2F5}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9DACD6FB-C686-417D-A8B1-50AEF392D0E3}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E6D8C8AD-1B56-488A-B60F-B98CA70300CF}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{20A8CCBE-0636-46B6-969A-000D58572033}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7A2A925D-DDD1-45EA-AF54-F15AA80C8379}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7AA6BB59-FD1A-45B3-8899-746BAF81E399}"/>
 </file>
</xml_diff>

<commit_message>
Actualizacao da leitura dos graficos na pagina geral
</commit_message>
<xml_diff>
--- a/log_acoes.xlsx
+++ b/log_acoes.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C32"/>
+  <dimension ref="A1:C34"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -895,6 +895,40 @@
       <c r="C32" t="inlineStr">
         <is>
           <t>2026-04-17 10:21:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Atualizou os dados</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>2026-04-20 10:07:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Atualizou os dados</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>2026-04-21 09:55:48</t>
         </is>
       </c>
     </row>
@@ -1159,13 +1193,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4A5DA93F-8B64-4C25-85FB-BFB34D700397}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C168C831-AFAB-4CD0-98E8-0266DAD6668D}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B94FB21F-4D69-46DF-81F1-3B30EF5C181C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{30962EE3-5E68-4682-966F-8026FA6C05DF}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{895A2B9E-620C-4DD5-9D70-61A26072FEFB}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B2A099F0-23CC-4342-97FA-7DF1EF9B01A2}"/>
 </file>
</xml_diff>

<commit_message>
Actualizacao dos textos de leitura e interpretacao dos graficos
</commit_message>
<xml_diff>
--- a/log_acoes.xlsx
+++ b/log_acoes.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C34"/>
+  <dimension ref="A1:C37"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -929,6 +929,57 @@
       <c r="C34" t="inlineStr">
         <is>
           <t>2026-04-21 09:55:48</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Atualizou os dados</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>2026-04-23 10:20:16</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Atualizou os dados</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>2026-04-23 14:34:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Atualizou os dados</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>2026-04-23 14:52:50</t>
         </is>
       </c>
     </row>
@@ -1193,13 +1244,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C168C831-AFAB-4CD0-98E8-0266DAD6668D}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{95318E3B-2482-42F2-99FF-14E889686836}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{30962EE3-5E68-4682-966F-8026FA6C05DF}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B50BF38B-926D-4F8D-A0CD-B1BA04D85A68}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B2A099F0-23CC-4342-97FA-7DF1EF9B01A2}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B5559005-973C-447D-ADF7-DA9E2F709660}"/>
 </file>
</xml_diff>

<commit_message>
Actualizacao das presencas individuais
</commit_message>
<xml_diff>
--- a/log_acoes.xlsx
+++ b/log_acoes.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:C39"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -980,6 +980,40 @@
       <c r="C37" t="inlineStr">
         <is>
           <t>2026-04-23 14:52:50</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Atualizou os dados</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>2026-04-27 14:48:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Atualizou os dados</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>2026-04-29 14:41:14</t>
         </is>
       </c>
     </row>
@@ -1244,13 +1278,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{95318E3B-2482-42F2-99FF-14E889686836}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{02996B80-3846-410F-AB41-8AB935EEFB55}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B50BF38B-926D-4F8D-A0CD-B1BA04D85A68}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{05B91477-704C-4F02-8C96-75E69CFCD842}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B5559005-973C-447D-ADF7-DA9E2F709660}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CA97A402-2DF9-4365-8542-AC9011575AD6}"/>
 </file>
</xml_diff>

<commit_message>
Actuazacao das 12 sessoes
</commit_message>
<xml_diff>
--- a/log_acoes.xlsx
+++ b/log_acoes.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C39"/>
+  <dimension ref="A1:C41"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -1017,274 +1017,41 @@
         </is>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Atualizou os dados</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>2026-05-04 08:47:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Atualizou os dados</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>2026-05-04 11:42:40</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100DC8BB5B596CFDD4794B3344F0E8F53A4" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="481cb719fb2f51215cc00c8d40533043">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="20d57abc-823c-4051-a81a-1a0a01a8f39e" xmlns:ns3="54c5ab46-7543-4aba-b0fa-79d6a199bef5" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="71df0815368817fe9627576b1e062219" ns2:_="" ns3:_="">
-    <xsd:import namespace="20d57abc-823c-4051-a81a-1a0a01a8f39e"/>
-    <xsd:import namespace="54c5ab46-7543-4aba-b0fa-79d6a199bef5"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="20d57abc-823c-4051-a81a-1a0a01a8f39e" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="14" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="15" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="16" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="17" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="edc6e55a-975c-4e83-894d-449406ca2714" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="22" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="54c5ab46-7543-4aba-b0fa-79d6a199bef5" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="SharedWithUsers" ma:index="12" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:UserMulti">
-            <xsd:sequence>
-              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
-                <xsd:complexType>
-                  <xsd:sequence>
-                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
-                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
-                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
-                  </xsd:sequence>
-                </xsd:complexType>
-              </xsd:element>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="13" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{21a739d7-e82a-41d6-a891-a689fdcdcba6}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="54c5ab46-7543-4aba-b0fa-79d6a199bef5">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="54c5ab46-7543-4aba-b0fa-79d6a199bef5" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="20d57abc-823c-4051-a81a-1a0a01a8f39e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{02996B80-3846-410F-AB41-8AB935EEFB55}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{05B91477-704C-4F02-8C96-75E69CFCD842}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CA97A402-2DF9-4365-8542-AC9011575AD6}"/>
 </file>
</xml_diff>